<commit_message>
feat: add InLineQC report template and associated excel mapping configuration
</commit_message>
<xml_diff>
--- a/data/templates/BaoCao_InLineQC_All_1780023089422.xlsx
+++ b/data/templates/BaoCao_InLineQC_All_1780023089422.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755884B9-FA0B-435A-80C6-6DDFFE068A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DCDF95F-6F0F-4DFB-B81B-C0200FAE214E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Báo cáo QC" sheetId="1" r:id="rId1"/>
@@ -152,8 +152,8 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -220,9 +220,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -237,9 +234,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -621,76 +621,76 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" customWidth="1"/>
+    <col min="3" max="3" width="6.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.33203125" customWidth="1"/>
+    <col min="5" max="5" width="28.36328125" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="26.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:10" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="13" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="13"/>
-    </row>
-    <row r="3" spans="1:10" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J1" s="12"/>
+    </row>
+    <row r="3" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
       <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10"/>
+      <c r="F4" s="9"/>
       <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="10"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I4" s="9"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+    </row>
+    <row r="6" spans="1:10" ht="28" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -722,7 +722,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="5"/>
       <c r="C7" s="4"/>
@@ -734,7 +734,7 @@
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="5"/>
       <c r="C8" s="4"/>
@@ -746,19 +746,19 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="13"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="4"/>
@@ -770,19 +770,19 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="4"/>
@@ -794,19 +794,19 @@
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="5"/>
       <c r="C14" s="4"/>
@@ -818,7 +818,7 @@
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="5"/>
       <c r="C15" s="4"/>
@@ -830,33 +830,33 @@
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="13"/>
       <c r="B16" s="5"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
feat: implement excel report service and template filler with comprehensive unit tests
</commit_message>
<xml_diff>
--- a/data/templates/BaoCao_InLineQC_All_1780023089422.xlsx
+++ b/data/templates/BaoCao_InLineQC_All_1780023089422.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DCDF95F-6F0F-4DFB-B81B-C0200FAE214E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A03034E-B589-4AB2-9829-326989DCD161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -202,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -220,6 +220,9 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -235,7 +238,7 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -636,59 +639,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="11" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="12" t="s">
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="12"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
       <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="9"/>
+      <c r="F4" s="10"/>
       <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="9"/>
+      <c r="I4" s="10"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
     </row>
     <row r="6" spans="1:10" ht="28" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -725,43 +728,42 @@
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="5"/>
-      <c r="C7" s="4"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="4"/>
       <c r="E7" s="3"/>
       <c r="F7" s="4"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
-      <c r="I7" s="5"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="5"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="5"/>
-      <c r="C8" s="4"/>
+      <c r="C8" s="3"/>
       <c r="D8" s="4"/>
       <c r="E8" s="3"/>
       <c r="F8" s="4"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="13"/>
+      <c r="A9" s="7"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="5"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="3"/>
       <c r="J9" s="5"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
+      <c r="C10" s="3"/>
       <c r="D10" s="4"/>
       <c r="E10" s="3"/>
       <c r="F10" s="4"/>
@@ -771,21 +773,21 @@
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
-      <c r="C12" s="4"/>
+      <c r="C12" s="3"/>
       <c r="D12" s="4"/>
       <c r="E12" s="3"/>
       <c r="F12" s="4"/>
@@ -795,68 +797,68 @@
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="5"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="3"/>
       <c r="D14" s="4"/>
       <c r="E14" s="3"/>
       <c r="F14" s="4"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="I14" s="5"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="5"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="5"/>
-      <c r="C15" s="4"/>
+      <c r="C15" s="3"/>
       <c r="D15" s="4"/>
       <c r="E15" s="3"/>
       <c r="F15" s="4"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="5"/>
+      <c r="I15" s="3"/>
       <c r="J15" s="5"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="13"/>
+      <c r="A16" s="7"/>
       <c r="B16" s="5"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="5"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="3"/>
       <c r="J16" s="5"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
feat: implement Excel template filling service with data conversion and subtotal support
</commit_message>
<xml_diff>
--- a/data/templates/BaoCao_InLineQC_All_1780023089422.xlsx
+++ b/data/templates/BaoCao_InLineQC_All_1780023089422.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A03034E-B589-4AB2-9829-326989DCD161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F405D55-CF47-463C-B6D2-D5EF4D9FC0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -223,6 +223,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -236,9 +239,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -633,65 +633,65 @@
     <col min="5" max="5" width="28.36328125" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="14.08984375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="13" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="13"/>
+      <c r="J1" s="14"/>
     </row>
     <row r="3" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10"/>
+      <c r="F4" s="11"/>
       <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="10"/>
+      <c r="I4" s="11"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" spans="1:10" ht="28" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -752,7 +752,7 @@
       <c r="A9" s="7"/>
       <c r="B9" s="5"/>
       <c r="C9" s="7"/>
-      <c r="D9" s="14"/>
+      <c r="D9" s="8"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
@@ -776,7 +776,7 @@
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
-      <c r="D11" s="14"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
@@ -800,7 +800,7 @@
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
-      <c r="D13" s="14"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
@@ -836,7 +836,7 @@
       <c r="A16" s="7"/>
       <c r="B16" s="5"/>
       <c r="C16" s="7"/>
-      <c r="D16" s="14"/>
+      <c r="D16" s="8"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
@@ -845,20 +845,20 @@
       <c r="J16" s="5"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>